<commit_message>
Ajustando dados da planilha modelo
</commit_message>
<xml_diff>
--- a/src/test/resources/apartamento-modelo.xlsx
+++ b/src/test/resources/apartamento-modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicon\Documents\projects\nord-tool-backend\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52081A2A-43CE-4F29-9F3A-3469EACFA932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EDBB45C-EA42-4746-BC54-B61E68676865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4260" yWindow="1650" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
   <si>
     <t>Dia da Semana</t>
   </si>
@@ -68,9 +68,6 @@
   </si>
   <si>
     <t>agendado</t>
-  </si>
-  <si>
-    <t>teste</t>
   </si>
 </sst>
 </file>
@@ -486,7 +483,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -529,6 +526,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:H1 E2:F2 H2" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>